<commit_message>
Regenerate estimate demo against current engine + catalog
The committed demo predated this session's parse-bug catalog refresh (job counts
shifted, e.g. plumbing 42j->81j) and the price_scope unit-vs-lump fix. Regenerated
so the sample output matches the live engine.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/estimate_out.xlsx
+++ b/estimate_out.xlsx
@@ -2763,7 +2763,7 @@
       </c>
       <c r="D30" s="12" t="n"/>
       <c r="E30" s="14" t="n">
-        <v>1300</v>
+        <v>1225</v>
       </c>
       <c r="F30" s="14" t="n"/>
       <c r="G30" s="14" t="n"/>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="E57" s="14" t="n">
-        <v>8.9</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="F57" s="14" t="n"/>
       <c r="G57" s="14" t="n"/>
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="E58" s="14" t="n">
-        <v>7.25</v>
+        <v>6.5</v>
       </c>
       <c r="F58" s="14" t="n"/>
       <c r="G58" s="14" t="n"/>
@@ -4299,7 +4299,7 @@
         </is>
       </c>
       <c r="E62" s="14" t="n">
-        <v>3.21</v>
+        <v>2.35</v>
       </c>
       <c r="F62" s="14" t="n"/>
       <c r="G62" s="14" t="n"/>
@@ -4355,7 +4355,7 @@
         </is>
       </c>
       <c r="E63" s="14" t="n">
-        <v>3.75</v>
+        <v>3.25</v>
       </c>
       <c r="F63" s="14" t="n"/>
       <c r="G63" s="14" t="n"/>
@@ -6141,7 +6141,7 @@
         </is>
       </c>
       <c r="E99" s="14" t="n">
-        <v>3.12</v>
+        <v>1.85</v>
       </c>
       <c r="F99" s="14" t="n"/>
       <c r="G99" s="14" t="n"/>
@@ -6553,7 +6553,7 @@
         </is>
       </c>
       <c r="E107" s="14" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="F107" s="14" t="n"/>
       <c r="G107" s="14" t="n"/>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="E108" s="29" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F108" s="29" t="n"/>
       <c r="G108" s="29" t="n"/>
@@ -6661,7 +6661,7 @@
         </is>
       </c>
       <c r="E109" s="14" t="n">
-        <v>13.75</v>
+        <v>10</v>
       </c>
       <c r="F109" s="14" t="n"/>
       <c r="G109" s="14" t="n"/>
@@ -8827,7 +8827,7 @@
         </is>
       </c>
       <c r="E153" s="49" t="n">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="F153" s="29" t="n"/>
       <c r="G153" s="29" t="n"/>

</xml_diff>